<commit_message>
Отчёт 2026-03-23 13:00 MSK
</commit_message>
<xml_diff>
--- a/logs/excel/fedresurs_2026-03-23.xlsx
+++ b/logs/excel/fedresurs_2026-03-23.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>Компания не найдена</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>Компания не найдена</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -499,7 +499,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>Компания не найдена</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -517,12 +517,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Сведения о банкротстве:
-Публикации:
-- 10592731 от 10.01.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 04586390 от 09.12.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 04031970 от 24.06.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 03949602 от 27.05.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве</t>
+          <t>Компания не найдена</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -540,43 +535,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Сведения о банкротстве:
-Публикации:
-- 33724416 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 33724400 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 33724312 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 33724347 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 27696837 от 14.05.2025 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 27212505 от 23.04.2025 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 16349017 от 25.08.2023 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 14495468 от 01.02.2023 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 14160220 от 16.12.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 13970684 от 30.11.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 13629950 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 13607030 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 13630478 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 13441177 от 12.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 13441131 от 12.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 11223158 от 24.02.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 10314580 от 10.12.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 10069405 от 18.11.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 09924266 от 20.10.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 09755518 от 06.10.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 09708710 от 29.09.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 09242657 от 06.08.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 08703978 от 02.07.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 08704421 от 02.07.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 05799154 от 30.12.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 05704485 от 11.12.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 05616761 от 25.11.2020 Намерение должника обратиться в суд с заявлением о банкротстве
-- 05340350 от 14.10.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 05001697 от 25.06.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 04795597 от 19.03.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 04592154 от 12.12.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 03852906 от 22.04.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 03706767 от 25.02.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
-- 03196309 от 08.06.2018 Намерение должника обратиться в суд с заявлением о банкротстве
-- 00109989 от 19.08.2015 Намерение должника обратиться в суд с заявлением о банкротстве</t>
+          <t>Компания не найдена</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>

</xml_diff>

<commit_message>
Отчёт 2026-03-23 14:20 MSK
</commit_message>
<xml_diff>
--- a/logs/excel/fedresurs_2026-03-23.xlsx
+++ b/logs/excel/fedresurs_2026-03-23.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Компания не найдена</t>
+          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Компания не найдена</t>
+          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -499,7 +499,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Компания не найдена</t>
+          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -517,7 +517,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Компания не найдена</t>
+          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -535,7 +535,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Компания не найдена</t>
+          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>

</xml_diff>

<commit_message>
Отчёт 2026-03-23 14:29 MSK
</commit_message>
<xml_diff>
--- a/logs/excel/fedresurs_2026-03-23.xlsx
+++ b/logs/excel/fedresurs_2026-03-23.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
+          <t>Ошибка: name 'logger' is not defined</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
+          <t>Ошибка: name 'logger' is not defined</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -499,7 +499,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
+          <t>Ошибка: name 'logger' is not defined</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -517,7 +517,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
+          <t>Ошибка: name 'logger' is not defined</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -535,7 +535,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ошибка: 'FedresursBankruptcyChecker' object has no attribute 'max_retries'</t>
+          <t>Ошибка: name 'logger' is not defined</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>

</xml_diff>

<commit_message>
Отчёт 2026-03-23 14:44 MSK
</commit_message>
<xml_diff>
--- a/logs/excel/fedresurs_2026-03-23.xlsx
+++ b/logs/excel/fedresurs_2026-03-23.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ошибка: name 'logger' is not defined</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ошибка: name 'logger' is not defined</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -499,7 +499,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ошибка: name 'logger' is not defined</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -517,7 +517,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ошибка: name 'logger' is not defined</t>
+          <t>Сведения о банкротстве:
+Публикации:
+- 10592731 от 10.01.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04586390 от 09.12.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04031970 от 24.06.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03949602 от 27.05.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -535,7 +540,43 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ошибка: name 'logger' is not defined</t>
+          <t>Сведения о банкротстве:
+Публикации:
+- 33724416 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 33724400 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 33724312 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 33724347 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 27696837 от 14.05.2025 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 27212505 от 23.04.2025 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 16349017 от 25.08.2023 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 14495468 от 01.02.2023 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 14160220 от 16.12.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13970684 от 30.11.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13629950 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13607030 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13630478 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13441177 от 12.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13441131 от 12.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 11223158 от 24.02.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 10314580 от 10.12.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 10069405 от 18.11.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09924266 от 20.10.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09755518 от 06.10.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09708710 от 29.09.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09242657 от 06.08.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 08703978 от 02.07.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 08704421 от 02.07.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05799154 от 30.12.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05704485 от 11.12.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05616761 от 25.11.2020 Намерение должника обратиться в суд с заявлением о банкротстве
+- 05340350 от 14.10.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05001697 от 25.06.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04795597 от 19.03.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04592154 от 12.12.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03852906 от 22.04.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03706767 от 25.02.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03196309 от 08.06.2018 Намерение должника обратиться в суд с заявлением о банкротстве
+- 00109989 от 19.08.2015 Намерение должника обратиться в суд с заявлением о банкротстве</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>

</xml_diff>